<commit_message>
feat: add explicit IST pipeline completion timestamps across Dashboard, Futures, and Post-Market views
</commit_message>
<xml_diff>
--- a/Post_Market_Indexes_Validation.xlsx
+++ b/Post_Market_Indexes_Validation.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,28 +504,28 @@
         <v>24624.65</v>
       </c>
       <c r="D2" t="n">
-        <v>24533.5</v>
+        <v>24624.65</v>
       </c>
       <c r="E2" t="n">
-        <v>91.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>24677.6</v>
       </c>
       <c r="G2" t="n">
-        <v>24637.91</v>
+        <v>24702.19</v>
       </c>
       <c r="H2" t="n">
-        <v>39.69</v>
+        <v>-24.59</v>
       </c>
       <c r="I2" t="n">
         <v>24497.95</v>
       </c>
       <c r="J2" t="n">
-        <v>24468.76</v>
+        <v>24522.54</v>
       </c>
       <c r="K2" t="n">
-        <v>29.19</v>
+        <v>-24.59</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -538,59 +538,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.37</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BANK NIFTY</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>57739.95</v>
-      </c>
-      <c r="D3" t="n">
-        <v>57541.8</v>
-      </c>
-      <c r="E3" t="n">
-        <v>198.15</v>
-      </c>
-      <c r="F3" t="n">
-        <v>57931.85</v>
-      </c>
-      <c r="G3" t="n">
-        <v>57818.39</v>
-      </c>
-      <c r="H3" t="n">
-        <v>113.46</v>
-      </c>
-      <c r="I3" t="n">
-        <v>57456.35</v>
-      </c>
-      <c r="J3" t="n">
-        <v>57378.69</v>
-      </c>
-      <c r="K3" t="n">
-        <v>77.66</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>🎯 TARGET HIT</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -694,28 +642,28 @@
         <v>57739.95</v>
       </c>
       <c r="D2" t="n">
-        <v>57541.8</v>
+        <v>57739.95</v>
       </c>
       <c r="E2" t="n">
-        <v>198.15</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>57931.85</v>
       </c>
       <c r="G2" t="n">
-        <v>57818.39</v>
+        <v>57962.41</v>
       </c>
       <c r="H2" t="n">
-        <v>113.46</v>
+        <v>-30.56</v>
       </c>
       <c r="I2" t="n">
         <v>57456.35</v>
       </c>
       <c r="J2" t="n">
-        <v>57378.69</v>
+        <v>57486.91</v>
       </c>
       <c r="K2" t="n">
-        <v>77.66</v>
+        <v>-30.56</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -728,7 +676,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>